<commit_message>
chore: render master to the site root
</commit_message>
<xml_diff>
--- a/StructureDefinition-mii-ex-labor-interpretationsbeeinflussende-eigenschaft.xlsx
+++ b/StructureDefinition-mii-ex-labor-interpretationsbeeinflussende-eigenschaft.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2027.0.0-ballot.rc4</t>
+    <t>2027.0.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-14T07:11:51+00:00</t>
+    <t>2026-09-14T07:28:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>